<commit_message>
Mise à jour du fichier Excel via Shiny
</commit_message>
<xml_diff>
--- a/prod_result_ELE.xlsx
+++ b/prod_result_ELE.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t xml:space="preserve">ANNEE</t>
   </si>
@@ -384,6 +384,54 @@
   </si>
   <si>
     <t xml:space="preserve">2025-10-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-01-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-07-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-10-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028-01-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028-07-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028-10-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2029-01-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2029-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2029-07-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2029-10-01</t>
   </si>
   <si>
     <t xml:space="preserve">1996</t>
@@ -553,7 +601,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFA500"/>
+        <fgColor rgb="FFB8F0F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1608,6 +1656,86 @@
         <v>121</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1626,127 +1754,127 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1762,7 +1890,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2">
@@ -2258,34 +2386,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2">
@@ -2317,7 +2445,7 @@
         <v>98305.901770633</v>
       </c>
       <c r="J2" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3">
@@ -2349,7 +2477,7 @@
         <v>98496.6371262413</v>
       </c>
       <c r="J3" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4">
@@ -2381,7 +2509,7 @@
         <v>98878.1078374579</v>
       </c>
       <c r="J4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5">
@@ -2413,7 +2541,7 @@
         <v>99450.3139042828</v>
       </c>
       <c r="J5" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6">
@@ -2445,7 +2573,7 @@
         <v>100792.108283122</v>
       </c>
       <c r="J6" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -2477,7 +2605,7 @@
         <v>102428.499468021</v>
       </c>
       <c r="J7" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8">
@@ -2509,7 +2637,7 @@
         <v>104933.933504379</v>
       </c>
       <c r="J8" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9">
@@ -2541,7 +2669,7 @@
         <v>108308.410392197</v>
       </c>
       <c r="J9" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10">
@@ -2573,7 +2701,7 @@
         <v>112190.725732575</v>
       </c>
       <c r="J10" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11">
@@ -2605,7 +2733,7 @@
         <v>115256.855000773</v>
       </c>
       <c r="J11" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12">
@@ -2637,7 +2765,7 @@
         <v>117159.212204924</v>
       </c>
       <c r="J12" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13">
@@ -2669,7 +2797,7 @@
         <v>117897.797345027</v>
       </c>
       <c r="J13" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14">
@@ -2701,7 +2829,7 @@
         <v>117133.368329486</v>
       </c>
       <c r="J14" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15">
@@ -2733,7 +2861,7 @@
         <v>117232.636374173</v>
       </c>
       <c r="J15" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16">
@@ -2765,7 +2893,7 @@
         <v>117855.131515726</v>
       </c>
       <c r="J16" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17">
@@ -2797,7 +2925,7 @@
         <v>119000.853754147</v>
       </c>
       <c r="J17" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18">
@@ -2829,7 +2957,7 @@
         <v>119386.445138653</v>
       </c>
       <c r="J18" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19">
@@ -2861,7 +2989,7 @@
         <v>121997.417461443</v>
       </c>
       <c r="J19" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20">
@@ -2893,7 +3021,7 @@
         <v>125568.162526388</v>
       </c>
       <c r="J20" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21">
@@ -2925,7 +3053,7 @@
         <v>130098.680333488</v>
       </c>
       <c r="J21" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22">
@@ -2957,7 +3085,7 @@
         <v>134443.990381895</v>
       </c>
       <c r="J22" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23">
@@ -2989,7 +3117,7 @@
         <v>135821.090820615</v>
       </c>
       <c r="J23" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24">
@@ -3021,7 +3149,7 @@
         <v>133131.363884514</v>
       </c>
       <c r="J24" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25">
@@ -3053,7 +3181,7 @@
         <v>126374.809573592</v>
       </c>
       <c r="J25" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26">
@@ -3085,7 +3213,7 @@
         <v>114837.554256535</v>
       </c>
       <c r="J26" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27">
@@ -3117,7 +3245,7 @@
         <v>106853.813601966</v>
       </c>
       <c r="J27" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28">
@@ -3149,7 +3277,7 @@
         <v>101642.847415964</v>
       </c>
       <c r="J28" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29">
@@ -3181,7 +3309,7 @@
         <v>99204.655698529</v>
       </c>
       <c r="J29" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30">
@@ -3213,7 +3341,7 @@
         <v>99941.7387467669</v>
       </c>
       <c r="J30" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31">
@@ -3245,7 +3373,7 @@
         <v>99953.5380147034</v>
       </c>
       <c r="J31" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32">
@@ -3277,7 +3405,7 @@
         <v>99641.2008690946</v>
       </c>
       <c r="J32" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33">
@@ -3309,7 +3437,7 @@
         <v>99004.7273099403</v>
       </c>
       <c r="J33" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34">
@@ -3341,7 +3469,7 @@
         <v>97599.6109648742</v>
       </c>
       <c r="J34" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35">
@@ -3373,7 +3501,7 @@
         <v>97097.3494748307</v>
       </c>
       <c r="J35" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36">
@@ -3405,7 +3533,7 @@
         <v>97049.0813131942</v>
       </c>
       <c r="J36" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37">
@@ -3437,7 +3565,7 @@
         <v>97454.8064799647</v>
       </c>
       <c r="J37" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38">
@@ -3469,7 +3597,7 @@
         <v>98009.4762998598</v>
       </c>
       <c r="J38" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39">
@@ -3501,7 +3629,7 @@
         <v>98202.5533006986</v>
       </c>
       <c r="J39" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40">
@@ -3533,7 +3661,7 @@
         <v>97731.6563274671</v>
       </c>
       <c r="J40" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41">
@@ -3565,7 +3693,7 @@
         <v>96596.7853801654</v>
       </c>
       <c r="J41" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42">
@@ -3597,7 +3725,7 @@
         <v>94768.7914458169</v>
       </c>
       <c r="J42" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43">
@@ -3629,7 +3757,7 @@
         <v>93259.393193344</v>
       </c>
       <c r="J43" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="44">
@@ -3661,7 +3789,7 @@
         <v>92038.8884906441</v>
       </c>
       <c r="J44" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="45">
@@ -3693,7 +3821,7 @@
         <v>91107.2773377172</v>
       </c>
       <c r="J45" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46">
@@ -3725,7 +3853,7 @@
         <v>90116.5875838359</v>
       </c>
       <c r="J46" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="47">
@@ -3757,7 +3885,7 @@
         <v>89745.2510234823</v>
       </c>
       <c r="J47" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
     </row>
     <row r="48">
@@ -3789,7 +3917,7 @@
         <v>89642.8232910932</v>
       </c>
       <c r="J48" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49">
@@ -3821,7 +3949,7 @@
         <v>89809.3043866686</v>
       </c>
       <c r="J49" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="50">
@@ -3853,7 +3981,7 @@
         <v>89767.7524814593</v>
       </c>
       <c r="J50" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="51">
@@ -3885,7 +4013,7 @@
         <v>90151.8761675345</v>
       </c>
       <c r="J51" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="52">
@@ -3917,7 +4045,7 @@
         <v>90487.0346452298</v>
       </c>
       <c r="J52" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="53">
@@ -3949,7 +4077,7 @@
         <v>90773.2279145451</v>
       </c>
       <c r="J53" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="54">
@@ -3981,7 +4109,7 @@
         <v>90479.0777362292</v>
       </c>
       <c r="J54" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="55">
@@ -4013,7 +4141,7 @@
         <v>90112.5844207433</v>
       </c>
       <c r="J55" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="56">
@@ -4045,7 +4173,7 @@
         <v>89143.7548205596</v>
       </c>
       <c r="J56" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="57">
@@ -4077,7 +4205,7 @@
         <v>87572.588935678</v>
       </c>
       <c r="J57" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="58">
@@ -4109,7 +4237,7 @@
         <v>84747.4810876344</v>
       </c>
       <c r="J58" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="59">
@@ -4141,7 +4269,7 @@
         <v>83307.9982217896</v>
       </c>
       <c r="J59" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60">
@@ -4173,7 +4301,7 @@
         <v>82585.9505671617</v>
       </c>
       <c r="J60" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61">
@@ -4205,7 +4333,7 @@
         <v>82581.3381237507</v>
       </c>
       <c r="J61" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62">
@@ -4237,7 +4365,7 @@
         <v>84575.6949835908</v>
       </c>
       <c r="J62" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="63">
@@ -4269,7 +4397,7 @@
         <v>85011.6809668716</v>
       </c>
       <c r="J63" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64">
@@ -4301,7 +4429,7 @@
         <v>85159.8629301242</v>
       </c>
       <c r="J64" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65">
@@ -4333,7 +4461,7 @@
         <v>85020.2408733487</v>
       </c>
       <c r="J65" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="66">
@@ -4365,7 +4493,7 @@
         <v>85882.9841431892</v>
       </c>
       <c r="J66" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
     </row>
     <row r="67">
@@ -4397,7 +4525,7 @@
         <v>86761.3141856383</v>
       </c>
       <c r="J67" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="68">
@@ -4429,7 +4557,7 @@
         <v>88951.9192464167</v>
       </c>
       <c r="J68" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="69">
@@ -4461,7 +4589,7 @@
         <v>92454.7993255243</v>
       </c>
       <c r="J69" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="70">
@@ -4493,7 +4621,7 @@
         <v>96980.534088626</v>
       </c>
       <c r="J70" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="71">
@@ -4525,7 +4653,7 @@
         <v>97345.5816371275</v>
       </c>
       <c r="J71" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72">
@@ -4557,7 +4685,7 @@
         <v>93274.8488131218</v>
       </c>
       <c r="J72" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="73">
@@ -4589,7 +4717,7 @@
         <v>84768.3356166089</v>
       </c>
       <c r="J73" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="74">
@@ -4621,7 +4749,7 @@
         <v>77341.3619563375</v>
       </c>
       <c r="J74" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="75">
@@ -4653,7 +4781,7 @@
         <v>68649.1788061499</v>
       </c>
       <c r="J75" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="76">
@@ -4685,7 +4813,7 @@
         <v>65200.9084249061</v>
       </c>
       <c r="J76" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="77">
@@ -4717,7 +4845,7 @@
         <v>66996.5508126062</v>
       </c>
       <c r="J77" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="78">
@@ -4749,7 +4877,7 @@
         <v>68413.7674234709</v>
       </c>
       <c r="J78" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="79">
@@ -4781,7 +4909,7 @@
         <v>72382.3475950667</v>
       </c>
       <c r="J79" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
     </row>
     <row r="80">
@@ -4813,7 +4941,7 @@
         <v>73814.5400857979</v>
       </c>
       <c r="J80" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="81">
@@ -4845,7 +4973,7 @@
         <v>72710.3448956643</v>
       </c>
       <c r="J81" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="82">
@@ -4877,7 +5005,7 @@
         <v>86589.948056443</v>
       </c>
       <c r="J82" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="83">
@@ -4909,7 +5037,7 @@
         <v>83126.4790588204</v>
       </c>
       <c r="J83" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
     </row>
     <row r="84">
@@ -4941,7 +5069,7 @@
         <v>80763.5915605545</v>
       </c>
       <c r="J84" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
     </row>
     <row r="85">
@@ -4973,7 +5101,7 @@
         <v>79501.2855616453</v>
       </c>
       <c r="J85" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="86">
@@ -5005,7 +5133,7 @@
         <v>74806.9817794573</v>
       </c>
       <c r="J86" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87">
@@ -5037,7 +5165,7 @@
         <v>75227.461587057</v>
       </c>
       <c r="J87" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="88">
@@ -5069,7 +5197,7 @@
         <v>76220.9065642795</v>
       </c>
       <c r="J88" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
     </row>
     <row r="89">
@@ -5101,7 +5229,7 @@
         <v>77787.316711125</v>
       </c>
       <c r="J89" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="90">
@@ -5133,7 +5261,7 @@
         <v>79926.6920275933</v>
       </c>
       <c r="J90" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
     </row>
     <row r="91">
@@ -5165,7 +5293,7 @@
         <v>81394.8576027545</v>
       </c>
       <c r="J91" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="92">
@@ -5197,7 +5325,7 @@
         <v>82191.8134366085</v>
       </c>
       <c r="J92" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="93">
@@ -5229,7 +5357,7 @@
         <v>82317.5595291554</v>
       </c>
       <c r="J93" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="94">
@@ -5261,7 +5389,7 @@
         <v>81772.0958803952</v>
       </c>
       <c r="J94" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="95">
@@ -5293,7 +5421,7 @@
         <v>81362.9981438251</v>
       </c>
       <c r="J95" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
     </row>
     <row r="96">
@@ -5325,7 +5453,7 @@
         <v>81090.2663194449</v>
       </c>
       <c r="J96" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="97">
@@ -5357,7 +5485,7 @@
         <v>80953.9004072549</v>
       </c>
       <c r="J97" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -5373,10 +5501,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2">
@@ -6305,6 +6433,134 @@
       </c>
       <c r="B117" t="n">
         <v>81221.0782166526</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>122</v>
+      </c>
+      <c r="B118" t="n">
+        <v>81219.9014113683</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>123</v>
+      </c>
+      <c r="B119" t="n">
+        <v>81218.9810639936</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>124</v>
+      </c>
+      <c r="B120" t="n">
+        <v>81218.3588504082</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>125</v>
+      </c>
+      <c r="B121" t="n">
+        <v>81218.0605053283</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>126</v>
+      </c>
+      <c r="B122" t="n">
+        <v>81218.4985655674</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123" t="n">
+        <v>81218.8412464683</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>128</v>
+      </c>
+      <c r="B124" t="n">
+        <v>81219.0729395152</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125" t="n">
+        <v>81219.1840065021</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>130</v>
+      </c>
+      <c r="B126" t="n">
+        <v>81219.0206704133</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>131</v>
+      </c>
+      <c r="B127" t="n">
+        <v>81218.892910177</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>132</v>
+      </c>
+      <c r="B128" t="n">
+        <v>81218.8065318091</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>133</v>
+      </c>
+      <c r="B129" t="n">
+        <v>81218.765120505</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>134</v>
+      </c>
+      <c r="B130" t="n">
+        <v>81218.8259830178</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>135</v>
+      </c>
+      <c r="B131" t="n">
+        <v>81218.873591026</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>136</v>
+      </c>
+      <c r="B132" t="n">
+        <v>81218.9057790775</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>137</v>
+      </c>
+      <c r="B133" t="n">
+        <v>81218.9212100127</v>
       </c>
     </row>
   </sheetData>
@@ -6320,10 +6576,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2">
@@ -7252,6 +7508,134 @@
       </c>
       <c r="B117" t="n">
         <v>81221.0782166526</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s">
+        <v>122</v>
+      </c>
+      <c r="B118" t="n">
+        <v>81219.9014113683</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s">
+        <v>123</v>
+      </c>
+      <c r="B119" t="n">
+        <v>81218.9810639936</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s">
+        <v>124</v>
+      </c>
+      <c r="B120" t="n">
+        <v>81218.3588504082</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s">
+        <v>125</v>
+      </c>
+      <c r="B121" t="n">
+        <v>81218.0605053283</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>126</v>
+      </c>
+      <c r="B122" t="n">
+        <v>81218.4985655674</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123" t="n">
+        <v>81218.8412464683</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s">
+        <v>128</v>
+      </c>
+      <c r="B124" t="n">
+        <v>81219.0729395152</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125" t="n">
+        <v>81219.1840065021</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s">
+        <v>130</v>
+      </c>
+      <c r="B126" t="n">
+        <v>81219.0206704133</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s">
+        <v>131</v>
+      </c>
+      <c r="B127" t="n">
+        <v>81218.892910177</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
+        <v>132</v>
+      </c>
+      <c r="B128" t="n">
+        <v>81218.8065318091</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>133</v>
+      </c>
+      <c r="B129" t="n">
+        <v>81218.765120505</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s">
+        <v>134</v>
+      </c>
+      <c r="B130" t="n">
+        <v>81218.8259830178</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s">
+        <v>135</v>
+      </c>
+      <c r="B131" t="n">
+        <v>81218.873591026</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s">
+        <v>136</v>
+      </c>
+      <c r="B132" t="n">
+        <v>81218.9057790775</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s">
+        <v>137</v>
+      </c>
+      <c r="B133" t="n">
+        <v>81218.9212100127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>